<commit_message>
Refresh the offline frontend snapshot for the foundation rules
The snapshot export that ran while adding the foundation rules aborted on a YAML
quoting error in the new file, and its failure was easy to miss in the combined
output, so the snapshot was left stale. CI checks it with
export_frontend_fixtures.py --check --grid-step 10, which now passes.
</commit_message>
<xml_diff>
--- a/frontend/src/mocks/fixtures/demo-import.xlsx
+++ b/frontend/src/mocks/fixtures/demo-import.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1570,7 +1570,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>超限不规则项</t>
+          <t>基础形式</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -1580,46 +1580,71 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>凹凸不规则,局部不规则</t>
+          <t>桩筏基础</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>桩基础</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>桩筏基础</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>桩筏基础</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>扭转不规则</t>
+          <t>桩基础</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>irregularity_items</t>
+          <t>foundation_type</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>【施工与安全】</t>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>地基基础工作年限</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>70</v>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" t="n">
+        <v>50</v>
+      </c>
+      <c r="F30" t="n">
+        <v>50</v>
+      </c>
+      <c r="G30" t="n">
+        <v>50</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>foundation_working_life</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>标准层重复率</t>
+          <t>超限不规则项</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -1627,63 +1652,48 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D31" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E31" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.75</v>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>凹凸不规则,局部不规则</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>扭转不规则</t>
+        </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>std_floor_repeat</t>
+          <t>irregularity_items</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>预制构件种类</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>种</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>20</v>
-      </c>
-      <c r="D32" t="n">
-        <v>14</v>
-      </c>
-      <c r="E32" t="n">
-        <v>8</v>
-      </c>
-      <c r="F32" t="n">
-        <v>12</v>
-      </c>
-      <c r="G32" t="n">
-        <v>15</v>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>component_types</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>【施工与安全】</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>风险特征</t>
+          <t>标准层重复率</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -1691,147 +1701,137 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>大悬挑,高支模</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>大悬挑,复杂地质</t>
-        </is>
+      <c r="C33" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.75</v>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>risk_features</t>
+          <t>std_floor_repeat</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>基坑开挖深度</t>
+          <t>预制构件种类</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>种</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4.5</v>
+        <v>20</v>
       </c>
       <c r="D34" t="n">
-        <v>4.5</v>
+        <v>14</v>
       </c>
       <c r="E34" t="n">
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="G34" t="n">
-        <v>4.5</v>
+        <v>15</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>excavation_depth</t>
+          <t>component_types</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>模板支撑高度</t>
+          <t>风险特征</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D35" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E35" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F35" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G35" t="n">
-        <v>4.5</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>大悬挑,高支模</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>大悬挑,复杂地质</t>
+        </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>formwork_height</t>
+          <t>risk_features</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>脚手架形式</t>
+          <t>基坑开挖深度</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>附着式升降脚手架</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>落地式钢管脚手架</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>附着式升降脚手架</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>附着式升降脚手架</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>附着式升降脚手架</t>
-        </is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G36" t="n">
+        <v>4.5</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>scaffold_type</t>
+          <t>excavation_depth</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>脚手架搭设高度</t>
+          <t>模板支撑高度</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1840,92 +1840,237 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>52.8</v>
+        <v>4.5</v>
       </c>
       <c r="D37" t="n">
-        <v>49</v>
+        <v>4.5</v>
       </c>
       <c r="E37" t="n">
-        <v>54</v>
+        <v>4.5</v>
       </c>
       <c r="F37" t="n">
-        <v>51</v>
+        <v>4.5</v>
       </c>
       <c r="G37" t="n">
-        <v>51</v>
+        <v>4.5</v>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>scaffold_height</t>
+          <t>formwork_height</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>【绿色低碳】</t>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>脚手架形式</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>落地式钢管脚手架</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>scaffold_type</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>预估装配率</t>
+          <t>脚手架搭设高度</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.25</v>
+        <v>52.8</v>
       </c>
       <c r="D39" t="n">
-        <v>0.45</v>
+        <v>49</v>
       </c>
       <c r="E39" t="n">
-        <v>0.75</v>
+        <v>54</v>
       </c>
       <c r="F39" t="n">
-        <v>0.5</v>
+        <v>51</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3</v>
+        <v>51</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>prefab_ratio_est</t>
+          <t>scaffold_height</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
+          <t>基坑支护形式</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>放坡开挖</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>地下连续墙</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>retaining_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>支护混凝土强度等级</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>30</v>
+      </c>
+      <c r="E41" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" t="n">
+        <v>30</v>
+      </c>
+      <c r="G41" t="n">
+        <v>25</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>retaining_concrete_grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>【绿色低碳】</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>预估装配率</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>prefab_ratio_est</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
           <t>绿地率</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C44" t="n">
         <v>0.38</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D44" t="n">
         <v>0.35</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E44" t="n">
         <v>0.36</v>
       </c>
-      <c r="F40" t="n">
+      <c r="F44" t="n">
         <v>0.4</v>
       </c>
-      <c r="G40" t="n">
+      <c r="G44" t="n">
         <v>0.35</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>green_ratio</t>
         </is>
@@ -1934,12 +2079,12 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A32:H32"/>
   </mergeCells>
-  <dataValidations count="30">
+  <dataValidations count="34">
     <dataValidation sqref="C3:H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【结构体系】必须是下列之一：剪力墙, 框架-剪力墙, 框架, 钢结构, MiC" type="list">
       <formula1>"剪力墙","框架-剪力墙","框架","钢结构","MiC"</formula1>
     </dataValidation>
@@ -2026,34 +2171,48 @@
       <formula1>0</formula1>
       <formula2>1e+308</formula2>
     </dataValidation>
-    <dataValidation sqref="C31:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【标准层重复率】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C32:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预制构件种类】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C34:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑开挖深度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C35:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【模板支撑高度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C36:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【脚手架形式】必须是下列之一：落地式钢管脚手架, 附着式升降脚手架, 悬挑式脚手架" type="list">
+    <dataValidation sqref="C29:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基础形式】必须是下列之一：筏形基础, 桩筏基础, 独立基础, 条形基础, 桩基础" type="list">
+      <formula1>"筏形基础","桩筏基础","独立基础","条形基础","桩基础"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C30:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【地基基础工作年限】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C33:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【标准层重复率】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C34:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预制构件种类】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C36:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑开挖深度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C37:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【模板支撑高度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C38:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【脚手架形式】必须是下列之一：落地式钢管脚手架, 附着式升降脚手架, 悬挑式脚手架" type="list">
       <formula1>"落地式钢管脚手架","附着式升降脚手架","悬挑式脚手架"</formula1>
     </dataValidation>
-    <dataValidation sqref="C37:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【脚手架搭设高度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C39:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预估装配率】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C40:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【绿地率】必须是数字" type="decimal" operator="between">
+    <dataValidation sqref="C39:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【脚手架搭设高度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C40:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基坑支护形式】必须是下列之一：排桩, 地下连续墙, 土钉墙, 放坡开挖, 其他" type="list">
+      <formula1>"排桩","地下连续墙","土钉墙","放坡开挖","其他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C41:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【支护混凝土强度等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C43:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预估装配率】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C44:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【绿地率】必须是数字" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1e+308</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Refresh the offline snapshot after the merge
The snapshot fingerprints the sources it was generated from, and evaluate.py
gained the signature fix after the last export, so CI's snapshot check failed
even though the branch was internally consistent. Re-exported; the check passes
again.
</commit_message>
<xml_diff>
--- a/frontend/src/mocks/fixtures/demo-import.xlsx
+++ b/frontend/src/mocks/fixtures/demo-import.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -655,11 +655,55 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>所在省份</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>项目所在省级行政区（两字母地区码，如 ZJ）。用于提示「所选的地方册是否与项目所在地一致」</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>province</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>适用标准册</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>适用的规则册；留空＝只用国家标准（GB）。GB 永远生效、不能去掉；加进省级地区码后，该省的地方规则才会参与评估</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>standard_packs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【用地面积】必须是数字" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1e+308</formula2>
@@ -681,6 +725,9 @@
     </dataValidation>
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【抗震设防烈度】必须是下列之一：6度(0.05g), 7度(0.10g)" type="list">
       <formula1>"6度(0.05g)","7度(0.10g)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【所在省份】必须是下列之一：BJ, TJ, HE, SX, NM, LN, JL, HL, SH, JS, ZJ, AH, FJ, JX, SD, HA, HB, HN, GD, GX, HI, CQ, SC, GZ, YN, XZ, SN, GS, QH, NX, XJ" type="list">
+      <formula1>"BJ","TJ","HE","SX","NM","LN","JL","HL","SH","JS","ZJ","AH","FJ","JX","SD","HA","HB","HN","GD","GX","HI","CQ","SC","GZ","YN","XZ","SN","GS","QH","NX","XJ"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -693,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1239,569 +1286,474 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>【结构与造价】</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>日照标准日</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>daylight_standard_day</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>总建筑面积</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>38400</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>40800</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>43200</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>40800</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>40800</v>
-      </c>
-      <c r="H19" s="5" t="n"/>
+          <t>居住空间总数</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>gfa</t>
+          <t>living_space_count</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>基底面积</t>
+          <t>满足日照空间数</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2400</v>
-      </c>
-      <c r="D20" t="n">
-        <v>2400</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2400</v>
-      </c>
-      <c r="F20" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G20" t="n">
-        <v>2400</v>
+          <t>个</t>
+        </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>footprint</t>
+          <t>daylight_room_count</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>楼栋数</t>
+          <t>室内净高</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>栋</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" t="n">
-        <v>4</v>
-      </c>
-      <c r="G21" t="n">
-        <v>4</v>
+          <t>m</t>
+        </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>buildings</t>
+          <t>clear_height</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>层数</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>层</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="H22" s="5" t="n"/>
+          <t>设新风/中央空调</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>floors</t>
+          <t>has_fresh_air</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>外表面积</t>
+          <t>设担架电梯</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D23" t="n">
-        <v>13200</v>
-      </c>
-      <c r="E23" t="n">
-        <v>14400</v>
-      </c>
-      <c r="F23" t="n">
-        <v>13000</v>
-      </c>
-      <c r="G23" t="n">
-        <v>14000</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>envelope_area</t>
+          <t>has_stretcher_elevator</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>建筑体积</t>
+          <t>设无障碍电梯</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>126720</v>
-      </c>
-      <c r="D24" t="n">
-        <v>118320</v>
-      </c>
-      <c r="E24" t="n">
-        <v>129600</v>
-      </c>
-      <c r="F24" t="n">
-        <v>122400</v>
-      </c>
-      <c r="G24" t="n">
-        <v>122400</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>volume</t>
+          <t>has_accessible_elevator</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>楼板厚度</t>
+          <t>电梯总台数</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>120</v>
-      </c>
-      <c r="D25" t="n">
-        <v>100</v>
-      </c>
-      <c r="E25" t="n">
-        <v>120</v>
-      </c>
-      <c r="F25" t="n">
-        <v>120</v>
-      </c>
-      <c r="G25" t="n">
-        <v>110</v>
+          <t>台</t>
+        </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>slab_thickness</t>
+          <t>total_elevators</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>结构设计工作年限</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>年</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>70</v>
-      </c>
-      <c r="D26" t="n">
-        <v>50</v>
-      </c>
-      <c r="E26" t="n">
-        <v>50</v>
-      </c>
-      <c r="F26" t="n">
-        <v>50</v>
-      </c>
-      <c r="G26" t="n">
-        <v>50</v>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>design_working_life</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>【结构与造价】</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>最小平面宽度</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>16</v>
-      </c>
-      <c r="D27" t="n">
-        <v>15</v>
-      </c>
-      <c r="E27" t="n">
-        <v>16</v>
-      </c>
-      <c r="F27" t="n">
-        <v>16</v>
-      </c>
-      <c r="G27" t="n">
-        <v>14</v>
-      </c>
+          <t>总建筑面积</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>38400</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>40800</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>43200</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>40800</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>40800</v>
+      </c>
+      <c r="H27" s="5" t="n"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>min_plan_width</t>
+          <t>gfa</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>混凝土强度等级</t>
+          <t>基底面积</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30</v>
+        <v>2400</v>
       </c>
       <c r="D28" t="n">
-        <v>25</v>
+        <v>2400</v>
       </c>
       <c r="E28" t="n">
-        <v>30</v>
+        <v>2400</v>
       </c>
       <c r="F28" t="n">
-        <v>30</v>
+        <v>2400</v>
       </c>
       <c r="G28" t="n">
-        <v>25</v>
+        <v>2400</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>concrete_grade</t>
+          <t>footprint</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>结构高度分类</t>
+          <t>楼栋数</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>栋</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>structural_height_classification</t>
+          <t>buildings</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>基础形式</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>桩筏基础</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>桩基础</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>桩筏基础</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>桩筏基础</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>桩基础</t>
-        </is>
-      </c>
+          <t>层数</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>层</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="H30" s="5" t="n"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>foundation_type</t>
+          <t>floors</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>基础混凝土强度等级</t>
+          <t>外表面积</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>MPa</t>
-        </is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D31" t="n">
+        <v>13200</v>
+      </c>
+      <c r="E31" t="n">
+        <v>14400</v>
+      </c>
+      <c r="F31" t="n">
+        <v>13000</v>
+      </c>
+      <c r="G31" t="n">
+        <v>14000</v>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>foundation_concrete_grade</t>
+          <t>envelope_area</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>地基基础工作年限</t>
+          <t>建筑体积</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>年</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70</v>
+        <v>126720</v>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>118320</v>
       </c>
       <c r="E32" t="n">
-        <v>50</v>
+        <v>129600</v>
       </c>
       <c r="F32" t="n">
-        <v>50</v>
+        <v>122400</v>
       </c>
       <c r="G32" t="n">
-        <v>50</v>
+        <v>122400</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>foundation_working_life</t>
+          <t>volume</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>钢结构体系</t>
+          <t>楼板厚度</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>120</v>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="n">
+        <v>120</v>
+      </c>
+      <c r="F33" t="n">
+        <v>120</v>
+      </c>
+      <c r="G33" t="n">
+        <v>110</v>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>steel_system</t>
+          <t>slab_thickness</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>是否设地下室</t>
+          <t>结构设计工作年限</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>70</v>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+      <c r="E34" t="n">
+        <v>50</v>
+      </c>
+      <c r="F34" t="n">
+        <v>50</v>
+      </c>
+      <c r="G34" t="n">
+        <v>50</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>has_basement</t>
+          <t>design_working_life</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>剪力墙截面厚度</t>
+          <t>最小平面宽度</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>200</v>
+        <v>16</v>
       </c>
       <c r="D35" t="n">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="E35" t="n">
-        <v>200</v>
+        <v>16</v>
       </c>
       <c r="F35" t="n">
-        <v>200</v>
+        <v>16</v>
       </c>
       <c r="G35" t="n">
-        <v>200</v>
+        <v>14</v>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>shear_wall_thickness</t>
+          <t>min_plan_width</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>框架梁截面宽度</t>
+          <t>混凝土强度等级</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>MPa</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>250</v>
+        <v>30</v>
       </c>
       <c r="D36" t="n">
-        <v>250</v>
+        <v>25</v>
       </c>
       <c r="E36" t="n">
-        <v>250</v>
+        <v>30</v>
       </c>
       <c r="F36" t="n">
-        <v>250</v>
+        <v>30</v>
       </c>
       <c r="G36" t="n">
-        <v>250</v>
+        <v>25</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>frame_beam_width</t>
+          <t>concrete_grade</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>框架柱截面形状</t>
+          <t>结构高度分类</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1809,131 +1761,107 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>矩形</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>矩形</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>矩形</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>矩形</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>矩形</t>
-        </is>
-      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>frame_column_shape</t>
+          <t>structural_height_classification</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>框架柱截面尺寸</t>
+          <t>基础形式</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>400</v>
-      </c>
-      <c r="D38" t="n">
-        <v>400</v>
-      </c>
-      <c r="E38" t="n">
-        <v>400</v>
-      </c>
-      <c r="F38" t="n">
-        <v>400</v>
-      </c>
-      <c r="G38" t="n">
-        <v>400</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>桩筏基础</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>桩基础</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>桩筏基础</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>桩筏基础</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>桩基础</t>
+        </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>frame_column_size</t>
+          <t>foundation_type</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>筏基底板贯通筋配筋率</t>
+          <t>基础混凝土强度等级</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0.2</v>
+          <t>MPa</t>
+        </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>raft_rebar_ratio</t>
+          <t>foundation_concrete_grade</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>基础埋置深度</t>
+          <t>地基基础工作年限</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>年</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="D40" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="F40" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="G40" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>foundation_depth</t>
+          <t>foundation_working_life</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>是否存在错层</t>
+          <t>钢结构体系</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -1941,75 +1869,90 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>has_staggered_floor</t>
+          <t>steel_system</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>错层处构件混凝土等级</t>
+          <t>是否设地下室</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>staggered_concrete_grade</t>
+          <t>has_basement</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>错层处是否有平面外受力墙</t>
+          <t>剪力墙截面厚度</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>200</v>
+      </c>
+      <c r="D43" t="n">
+        <v>200</v>
+      </c>
+      <c r="E43" t="n">
+        <v>200</v>
+      </c>
+      <c r="F43" t="n">
+        <v>200</v>
+      </c>
+      <c r="G43" t="n">
+        <v>200</v>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>has_out_of_plane_staggered_wall</t>
+          <t>shear_wall_thickness</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>错层处平面外受力墙厚度</t>
+          <t>框架梁截面宽度</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -2017,16 +1960,31 @@
           <t>mm</t>
         </is>
       </c>
+      <c r="C44" t="n">
+        <v>250</v>
+      </c>
+      <c r="D44" t="n">
+        <v>250</v>
+      </c>
+      <c r="E44" t="n">
+        <v>250</v>
+      </c>
+      <c r="F44" t="n">
+        <v>250</v>
+      </c>
+      <c r="G44" t="n">
+        <v>250</v>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>staggered_wall_thickness</t>
+          <t>frame_beam_width</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>是否单跨框架</t>
+          <t>框架柱截面形状</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -2036,258 +1994,222 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>矩形</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>矩形</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>矩形</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>矩形</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>矩形</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>is_single_span_frame</t>
+          <t>frame_column_shape</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>超限不规则项</t>
+          <t>框架柱截面尺寸</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>凹凸不规则,局部不规则</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>扭转不规则</t>
-        </is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D46" t="n">
+        <v>400</v>
+      </c>
+      <c r="E46" t="n">
+        <v>400</v>
+      </c>
+      <c r="F46" t="n">
+        <v>400</v>
+      </c>
+      <c r="G46" t="n">
+        <v>400</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>irregularity_items</t>
+          <t>frame_column_size</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>【施工与安全】</t>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>筏基底板贯通筋配筋率</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>raft_rebar_ratio</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>标准层重复率</t>
+          <t>基础埋置深度</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.65</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
-        <v>0.8</v>
+        <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>0.95</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
-        <v>0.85</v>
+        <v>6</v>
       </c>
       <c r="G48" t="n">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>std_floor_repeat</t>
+          <t>foundation_depth</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>预制构件种类</t>
+          <t>是否存在错层</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>种</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>20</v>
-      </c>
-      <c r="D49" t="n">
-        <v>14</v>
-      </c>
-      <c r="E49" t="n">
-        <v>8</v>
-      </c>
-      <c r="F49" t="n">
-        <v>12</v>
-      </c>
-      <c r="G49" t="n">
-        <v>15</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>component_types</t>
+          <t>has_staggered_floor</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>风险特征</t>
+          <t>错层处构件混凝土等级</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>大悬挑,高支模</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>大悬挑,复杂地质</t>
+          <t>MPa</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>risk_features</t>
+          <t>staggered_concrete_grade</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>基坑开挖深度</t>
+          <t>错层处是否有平面外受力墙</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D51" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E51" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F51" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G51" t="n">
-        <v>4.5</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>excavation_depth</t>
+          <t>has_out_of_plane_staggered_wall</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>模板支撑高度</t>
+          <t>错层处平面外受力墙厚度</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D52" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E52" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F52" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G52" t="n">
-        <v>4.5</v>
+          <t>mm</t>
+        </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>formwork_height</t>
+          <t>staggered_wall_thickness</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>脚手架形式</t>
+          <t>是否单跨框架</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2297,113 +2219,88 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>附着式升降脚手架</t>
+          <t>否</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>落地式钢管脚手架</t>
+          <t>否</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>附着式升降脚手架</t>
+          <t>否</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>附着式升降脚手架</t>
+          <t>否</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>附着式升降脚手架</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>scaffold_type</t>
+          <t>is_single_span_frame</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>脚手架搭设高度</t>
+          <t>超限不规则项</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="D54" t="n">
-        <v>49</v>
-      </c>
-      <c r="E54" t="n">
-        <v>54</v>
-      </c>
-      <c r="F54" t="n">
-        <v>51</v>
-      </c>
-      <c r="G54" t="n">
-        <v>51</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>凹凸不规则,局部不规则</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>扭转不规则</t>
+        </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>scaffold_height</t>
+          <t>irregularity_items</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>基坑支护形式</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>排桩</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>放坡开挖</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>排桩</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>地下连续墙</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>排桩</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>retaining_type</t>
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>【施工与安全】</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>地下连续墙是否两墙合一</t>
+          <t>标准层重复率</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -2411,163 +2308,243 @@
           <t>—</t>
         </is>
       </c>
+      <c r="C56" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.75</v>
+      </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>retaining_wall_two_in_one</t>
+          <t>std_floor_repeat</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>支护混凝土强度等级</t>
+          <t>预制构件种类</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>种</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>30</v>
+        <v>20</v>
+      </c>
+      <c r="D57" t="n">
+        <v>14</v>
       </c>
       <c r="E57" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F57" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="G57" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>retaining_concrete_grade</t>
+          <t>component_types</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>基坑工作年限</t>
+          <t>风险特征</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>年</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" t="n">
-        <v>2</v>
-      </c>
-      <c r="E58" t="n">
-        <v>2</v>
-      </c>
-      <c r="F58" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" t="n">
-        <v>2</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>大悬挑,高支模</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>大悬挑,复杂地质</t>
+        </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>excavation_working_life</t>
+          <t>risk_features</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>内支撑 / 锚拉体系</t>
+          <t>基坑开挖深度</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>混凝土内支撑</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>无内支撑与锚拉</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>混凝土内支撑</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>锚杆（锚拉）</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>无内支撑与锚拉</t>
-        </is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D59" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E59" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F59" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G59" t="n">
+        <v>4.5</v>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>brace_type</t>
+          <t>excavation_depth</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>内支撑混凝土强度等级</t>
+          <t>模板支撑高度</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>MPa</t>
-        </is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D60" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E60" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F60" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G60" t="n">
+        <v>4.5</v>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>brace_concrete_grade</t>
+          <t>formwork_height</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>锚杆自由段长度</t>
+          <t>脚手架形式</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>落地式钢管脚手架</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>附着式升降脚手架</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>scaffold_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>脚手架搭设高度</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
           <t>m</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>6</v>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>anchor_free_length</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>【绿色低碳】</t>
+      <c r="C62" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="D62" t="n">
+        <v>49</v>
+      </c>
+      <c r="E62" t="n">
+        <v>54</v>
+      </c>
+      <c r="F62" t="n">
+        <v>51</v>
+      </c>
+      <c r="G62" t="n">
+        <v>51</v>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>scaffold_height</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>预估装配率</t>
+          <t>基坑支护形式</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -2575,54 +2552,277 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C63" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D63" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E63" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F63" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G63" t="n">
-        <v>0.3</v>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>放坡开挖</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>地下连续墙</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>排桩</t>
+        </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>prefab_ratio_est</t>
+          <t>retaining_type</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
+          <t>地下连续墙是否两墙合一</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>retaining_wall_two_in_one</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>支护混凝土强度等级</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>30</v>
+      </c>
+      <c r="E65" t="n">
+        <v>30</v>
+      </c>
+      <c r="F65" t="n">
+        <v>30</v>
+      </c>
+      <c r="G65" t="n">
+        <v>25</v>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>retaining_concrete_grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>基坑工作年限</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2</v>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>excavation_working_life</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>内支撑 / 锚拉体系</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>混凝土内支撑</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>无内支撑与锚拉</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>混凝土内支撑</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>锚杆（锚拉）</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>无内支撑与锚拉</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>brace_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>内支撑混凝土强度等级</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>brace_concrete_grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>锚杆自由段长度</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>6</v>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>anchor_free_length</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>【绿色低碳】</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>人均公共绿地</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>m²/人</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>per_capita_green</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>预估装配率</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>prefab_ratio_est</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
           <t>绿地率</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
         <v>0.38</v>
       </c>
-      <c r="D64" t="n">
+      <c r="D73" t="n">
         <v>0.35</v>
       </c>
-      <c r="E64" t="n">
+      <c r="E73" t="n">
         <v>0.36</v>
       </c>
-      <c r="F64" t="n">
+      <c r="F73" t="n">
         <v>0.4</v>
       </c>
-      <c r="G64" t="n">
+      <c r="G73" t="n">
         <v>0.35</v>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>green_ratio</t>
         </is>
@@ -2630,13 +2830,13 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A55:H55"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A47:H47"/>
   </mergeCells>
-  <dataValidations count="49">
+  <dataValidations count="55">
     <dataValidation sqref="C3:H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【结构体系】必须是下列之一：剪力墙, 框架-剪力墙, 框架, 钢结构, MiC" type="list">
       <formula1>"剪力墙","框架-剪力墙","框架","钢结构","MiC"</formula1>
     </dataValidation>
@@ -2683,144 +2883,167 @@
       <formula1>0</formula1>
       <formula2>1e+308</formula2>
     </dataValidation>
-    <dataValidation sqref="C19:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【总建筑面积】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C20:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基底面积】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C21:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【楼栋数】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C22:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【层数】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C23:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【外表面积】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C24:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【建筑体积】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C25:H25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【楼板厚度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C26:H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【结构设计工作年限】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C27:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【最小平面宽度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C28:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【混凝土强度等级】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C29:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【结构高度分类】必须是下列之一：高层, 多层" type="list">
+    <dataValidation sqref="C18:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【日照标准日】必须是下列之一：大寒日, 冬至日" type="list">
+      <formula1>"大寒日","冬至日"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【居住空间总数】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C20:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【满足日照空间数】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C21:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【室内净高】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C25:H25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【电梯总台数】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C27:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【总建筑面积】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C28:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基底面积】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C29:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【楼栋数】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C30:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【层数】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C31:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【外表面积】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C32:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【建筑体积】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C33:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【楼板厚度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C34:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【结构设计工作年限】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C35:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【最小平面宽度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C36:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【混凝土强度等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C37:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【结构高度分类】必须是下列之一：高层, 多层" type="list">
       <formula1>"高层","多层"</formula1>
     </dataValidation>
-    <dataValidation sqref="C30:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基础形式】必须是下列之一：筏形基础, 桩筏基础, 独立基础, 条形基础, 桩基础" type="list">
+    <dataValidation sqref="C38:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基础形式】必须是下列之一：筏形基础, 桩筏基础, 独立基础, 条形基础, 桩基础" type="list">
       <formula1>"筏形基础","桩筏基础","独立基础","条形基础","桩基础"</formula1>
     </dataValidation>
-    <dataValidation sqref="C31:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基础混凝土强度等级】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C32:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【地基基础工作年限】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C33:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【钢结构体系】必须是下列之一：框架, 框架-中心支撑, 框架-偏心支撑（延性墙板）, 筒体和巨型框架" type="list">
+    <dataValidation sqref="C39:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基础混凝土强度等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C40:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【地基基础工作年限】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C41:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【钢结构体系】必须是下列之一：框架, 框架-中心支撑, 框架-偏心支撑（延性墙板）, 筒体和巨型框架" type="list">
       <formula1>"框架","框架-中心支撑","框架-偏心支撑（延性墙板）","筒体和巨型框架"</formula1>
     </dataValidation>
-    <dataValidation sqref="C35:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【剪力墙截面厚度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C36:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【框架梁截面宽度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C37:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【框架柱截面形状】必须是下列之一：矩形, 圆形" type="list">
+    <dataValidation sqref="C43:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【剪力墙截面厚度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C44:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【框架梁截面宽度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C45:H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【框架柱截面形状】必须是下列之一：矩形, 圆形" type="list">
       <formula1>"矩形","圆形"</formula1>
     </dataValidation>
-    <dataValidation sqref="C38:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【框架柱截面尺寸】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C39:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【筏基底板贯通筋配筋率】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C40:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基础埋置深度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C42:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【错层处构件混凝土等级】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C44:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【错层处平面外受力墙厚度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C48:H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【标准层重复率】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C49:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预制构件种类】必须是数字" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C51:H51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑开挖深度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C52:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【模板支撑高度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C53:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【脚手架形式】必须是下列之一：落地式钢管脚手架, 附着式升降脚手架, 悬挑式脚手架" type="list">
+    <dataValidation sqref="C46:H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【框架柱截面尺寸】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C47:H47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【筏基底板贯通筋配筋率】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C48:H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基础埋置深度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C50:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【错层处构件混凝土等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C52:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【错层处平面外受力墙厚度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C56:H56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【标准层重复率】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C57:H57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预制构件种类】必须是数字" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C59:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑开挖深度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C60:H60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【模板支撑高度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C61:H61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【脚手架形式】必须是下列之一：落地式钢管脚手架, 附着式升降脚手架, 悬挑式脚手架" type="list">
       <formula1>"落地式钢管脚手架","附着式升降脚手架","悬挑式脚手架"</formula1>
     </dataValidation>
-    <dataValidation sqref="C54:H54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【脚手架搭设高度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C55:H55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基坑支护形式】必须是下列之一：排桩, 地下连续墙, 土钉墙, 放坡开挖, 其他" type="list">
+    <dataValidation sqref="C62:H62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【脚手架搭设高度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C63:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【基坑支护形式】必须是下列之一：排桩, 地下连续墙, 土钉墙, 放坡开挖, 其他" type="list">
       <formula1>"排桩","地下连续墙","土钉墙","放坡开挖","其他"</formula1>
     </dataValidation>
-    <dataValidation sqref="C57:H57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【支护混凝土强度等级】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C58:H58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑工作年限】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C59:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【内支撑 / 锚拉体系】必须是下列之一：混凝土内支撑, 钢支撑, 锚杆（锚拉）, 无内支撑与锚拉" type="list">
+    <dataValidation sqref="C65:H65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【支护混凝土强度等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C66:H66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【基坑工作年限】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C67:H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="【内支撑 / 锚拉体系】必须是下列之一：混凝土内支撑, 钢支撑, 锚杆（锚拉）, 无内支撑与锚拉" type="list">
       <formula1>"混凝土内支撑","钢支撑","锚杆（锚拉）","无内支撑与锚拉"</formula1>
     </dataValidation>
-    <dataValidation sqref="C60:H60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【内支撑混凝土强度等级】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C61:H61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【锚杆自由段长度】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C63:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预估装配率】必须是数字" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>1e+308</formula2>
-    </dataValidation>
-    <dataValidation sqref="C64:H64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【绿地率】必须是数字" type="decimal" operator="between">
+    <dataValidation sqref="C68:H68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【内支撑混凝土强度等级】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C69:H69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【锚杆自由段长度】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C71:H71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【人均公共绿地】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C72:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【预估装配率】必须是数字" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1e+308</formula2>
+    </dataValidation>
+    <dataValidation sqref="C73:H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="类型错误" error="【绿地率】必须是数字" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1e+308</formula2>
     </dataValidation>

</xml_diff>